<commit_message>
Tagetik : noms dépense = DEPENSE_ACQ/DEPENSE_MARQUE (vue + fichier démo)
Aligne V_SOCLE_KPI.sql et DEMO_SOCLE_2027BUD_V1.xlsx sur les noms réels du
dataset (DEPENSE_ACQ, DEPENSE_MARQUE au lieu de DEP_ACQ/DEP_MARQUE).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BCU7CjG5rh6esFZ9teHY6F
</commit_message>
<xml_diff>
--- a/eduservices/tagetik/DEMO_SOCLE_2027BUD_V1.xlsx
+++ b/eduservices/tagetik/DEMO_SOCLE_2027BUD_V1.xlsx
@@ -587,12 +587,12 @@
       </c>
       <c r="T1" s="3" t="inlineStr">
         <is>
-          <t>DEP_ACQ</t>
+          <t>DEPENSE_ACQ</t>
         </is>
       </c>
       <c r="U1" s="3" t="inlineStr">
         <is>
-          <t>DEP_MARQUE</t>
+          <t>DEPENSE_MARQUE</t>
         </is>
       </c>
     </row>

</xml_diff>